<commit_message>
committed @ 2025-10-16-075924-0500 by tychen@TYCMBA.local
</commit_message>
<xml_diff>
--- a/data/3420-2025-fall-quizzes/3420-2025-fall-py-review-01-PLAY.xlsx
+++ b/data/3420-2025-fall-quizzes/3420-2025-fall-py-review-01-PLAY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcn85/workspace/dsm/data/3420-2025-fall-quizzes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tychen/workspace/dsm/data/3420-2025-fall-quizzes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B918A6A-794D-D842-984B-C3E0C5C9A92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEA40C8-D75F-3049-A6D6-7DB66164AB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19220" yWindow="-1340" windowWidth="19220" windowHeight="20980" xr2:uid="{02943BD8-8D23-1D42-A928-8937731C9A90}"/>
+    <workbookView xWindow="-32100" yWindow="-2880" windowWidth="32100" windowHeight="20980" activeTab="1" xr2:uid="{02943BD8-8D23-1D42-A928-8937731C9A90}"/>
   </bookViews>
   <sheets>
     <sheet name="py-np-pd" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="60">
   <si>
     <t>name</t>
   </si>
@@ -208,16 +208,16 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Johnson</t>
-  </si>
-  <si>
-    <t>q</t>
-  </si>
-  <si>
     <t>Quinn, J.</t>
   </si>
   <si>
     <t>SUM</t>
+  </si>
+  <si>
+    <t>Quinn J.</t>
+  </si>
+  <si>
+    <t>percent</t>
   </si>
 </sst>
 </file>
@@ -600,8 +600,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{625988FA-08F2-5D4B-BCDA-BABB71AA94B0}">
-  <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A2:K24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
@@ -612,185 +612,151 @@
     <col min="7" max="7" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
         <v>47</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" t="s">
         <v>49</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>50</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F2" t="s">
         <v>51</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G2" t="s">
         <v>52</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H2" t="s">
         <v>53</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I2" t="s">
         <v>54</v>
       </c>
-      <c r="J1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D2">
-        <v>0.25</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>1.5</v>
-      </c>
-      <c r="G2">
-        <v>0.25</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <f>SUM(D2:I2)</f>
-        <v>2</v>
-      </c>
-      <c r="K2" s="2">
-        <f>J2/10</f>
-        <v>0.2</v>
+      <c r="J2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="G3">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
         <f>SUM(D3:I3)</f>
-        <v>2</v>
+        <v>7.5</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" ref="K3:K18" si="0">J3/10</f>
-        <v>0.2</v>
+        <f>J3/10</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <f>SUM(D4:I4)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K4" s="2">
-        <f t="shared" si="0"/>
-        <v>0.2</v>
+        <f>J4/10</f>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E5">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1.25</v>
+      </c>
+      <c r="H5">
         <v>1.75</v>
       </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0.25</v>
-      </c>
       <c r="I5">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="J5">
         <f>SUM(D5:I5)</f>
-        <v>2.25</v>
+        <v>8.25</v>
       </c>
       <c r="K5" s="2">
-        <f t="shared" si="0"/>
-        <v>0.22500000000000001</v>
+        <f>J5/10</f>
+        <v>0.82499999999999996</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -826,16 +792,16 @@
         <v>3.75</v>
       </c>
       <c r="K6" s="2">
-        <f t="shared" si="0"/>
+        <f>J6/10</f>
         <v>0.375</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
@@ -844,7 +810,7 @@
         <v>1.75</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7">
         <v>2</v>
@@ -853,18 +819,18 @@
         <v>0.25</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <f>SUM(D7:I7)</f>
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="K7" s="2">
-        <f t="shared" si="0"/>
-        <v>0.4</v>
+        <f>J7/10</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -900,45 +866,45 @@
         <v>5.75</v>
       </c>
       <c r="K8" s="2">
-        <f t="shared" si="0"/>
+        <f>J8/10</f>
         <v>0.57499999999999996</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F9">
+        <v>1.5</v>
+      </c>
+      <c r="G9">
+        <v>1.5</v>
+      </c>
+      <c r="H9">
+        <v>0.5</v>
+      </c>
+      <c r="I9">
         <v>2</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>2</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
       </c>
       <c r="J9">
         <f>SUM(D9:I9)</f>
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="K9" s="2">
-        <f t="shared" si="0"/>
-        <v>0.6</v>
+        <f>J9/10</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -974,59 +940,59 @@
         <v>6.25</v>
       </c>
       <c r="K10" s="2">
-        <f t="shared" si="0"/>
+        <f>J10/10</f>
         <v>0.625</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D11">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="H11">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="I11">
         <v>2</v>
       </c>
       <c r="J11">
         <f>SUM(D11:I11)</f>
-        <v>6.75</v>
+        <v>12</v>
       </c>
       <c r="K11" s="2">
-        <f t="shared" si="0"/>
-        <v>0.67500000000000004</v>
+        <f>J11/10</f>
+        <v>1.2</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1038,409 +1004,447 @@
         <v>0.5</v>
       </c>
       <c r="H12">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <f>SUM(D12:I12)</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K12" s="2">
-        <f t="shared" si="0"/>
-        <v>0.7</v>
+        <f>J12/10</f>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D13">
-        <v>1.75</v>
+        <v>0.25</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G13">
         <v>0.25</v>
       </c>
       <c r="H13">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <f>SUM(D13:I13)</f>
-        <v>7.5</v>
+        <v>2</v>
       </c>
       <c r="K13" s="2">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
+        <f>J13/10</f>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14">
-        <v>2</v>
-      </c>
-      <c r="E14">
-        <v>2</v>
-      </c>
-      <c r="F14">
-        <v>1.75</v>
-      </c>
-      <c r="G14">
-        <v>1.25</v>
-      </c>
-      <c r="H14">
-        <v>0.5</v>
-      </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
-        <f>SUM(D14:I14)</f>
-        <v>7.5</v>
-      </c>
-      <c r="K14" s="2">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" t="s">
+        <v>55</v>
+      </c>
+      <c r="G14" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14" t="s">
+        <v>55</v>
+      </c>
+      <c r="I14" t="s">
+        <v>55</v>
+      </c>
+      <c r="J14" t="s">
+        <v>55</v>
+      </c>
+      <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15">
+        <v>1.75</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
         <v>2</v>
-      </c>
-      <c r="D15">
-        <v>2</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>1.5</v>
       </c>
       <c r="G15">
         <v>1.5</v>
       </c>
       <c r="H15">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J15">
         <f>SUM(D15:I15)</f>
-        <v>7.5</v>
+        <v>8.75</v>
       </c>
       <c r="K15" s="2">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
+        <f>J15/10</f>
+        <v>0.875</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16">
-        <v>1.5</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>2</v>
-      </c>
-      <c r="G16">
-        <v>1.25</v>
-      </c>
-      <c r="H16">
-        <v>1.75</v>
-      </c>
-      <c r="I16">
-        <v>1.75</v>
-      </c>
-      <c r="J16">
-        <f>SUM(D16:I16)</f>
-        <v>8.25</v>
-      </c>
-      <c r="K16" s="2">
-        <f t="shared" si="0"/>
-        <v>0.82499999999999996</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
+        <v>55</v>
+      </c>
+      <c r="F16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>55</v>
+      </c>
+      <c r="H16" t="s">
+        <v>55</v>
+      </c>
+      <c r="I16" t="s">
+        <v>55</v>
+      </c>
+      <c r="J16" t="s">
+        <v>55</v>
+      </c>
+      <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D17">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G17">
+        <v>0.5</v>
+      </c>
+      <c r="H17">
         <v>1.5</v>
-      </c>
-      <c r="H17">
-        <v>2</v>
       </c>
       <c r="I17">
         <v>1.5</v>
       </c>
       <c r="J17">
         <f>SUM(D17:I17)</f>
-        <v>8.75</v>
+        <v>7</v>
       </c>
       <c r="K17" s="2">
-        <f t="shared" si="0"/>
-        <v>0.875</v>
+        <f>J17/10</f>
+        <v>0.7</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="I18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J18">
         <f>SUM(D18:I18)</f>
-        <v>12</v>
+        <v>2.25</v>
       </c>
       <c r="K18" s="2">
-        <f t="shared" si="0"/>
-        <v>1.2</v>
+        <f>J18/10</f>
+        <v>0.22500000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G19" t="s">
-        <v>55</v>
-      </c>
-      <c r="H19" t="s">
-        <v>55</v>
-      </c>
-      <c r="I19" t="s">
-        <v>55</v>
-      </c>
-      <c r="J19" t="s">
-        <v>55</v>
-      </c>
-      <c r="K19" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="D19">
+        <v>0.5</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>1.5</v>
+      </c>
+      <c r="G19">
+        <v>1.25</v>
+      </c>
+      <c r="H19">
+        <v>1.5</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+      <c r="J19">
+        <f>SUM(D19:I19)</f>
+        <v>6.75</v>
+      </c>
+      <c r="K19" s="2">
+        <f>J19/10</f>
+        <v>0.67500000000000004</v>
+      </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" t="s">
-        <v>55</v>
-      </c>
-      <c r="E20" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" t="s">
-        <v>55</v>
-      </c>
-      <c r="G20" t="s">
-        <v>55</v>
-      </c>
-      <c r="H20" t="s">
-        <v>55</v>
-      </c>
-      <c r="I20" t="s">
-        <v>55</v>
-      </c>
-      <c r="J20" t="s">
-        <v>55</v>
-      </c>
-      <c r="K20" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="D20">
+        <v>0.5</v>
+      </c>
+      <c r="E20">
+        <v>0.5</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>2</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20">
+        <f>SUM(D20:I20)</f>
+        <v>6</v>
+      </c>
+      <c r="K20" s="2">
+        <f>J20/10</f>
+        <v>0.6</v>
+      </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" t="s">
+        <v>55</v>
+      </c>
+      <c r="G21" t="s">
+        <v>55</v>
+      </c>
+      <c r="H21" t="s">
+        <v>55</v>
+      </c>
+      <c r="I21" t="s">
+        <v>55</v>
+      </c>
+      <c r="J21" t="s">
+        <v>55</v>
+      </c>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>1.5</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0.5</v>
+      </c>
+      <c r="J22">
+        <f>SUM(D22:I22)</f>
+        <v>2</v>
+      </c>
+      <c r="K22" s="2">
+        <f>J22/10</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
         <v>57</v>
       </c>
-      <c r="D21" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" t="s">
-        <v>55</v>
-      </c>
-      <c r="G21" t="s">
-        <v>55</v>
-      </c>
-      <c r="H21" t="s">
-        <v>55</v>
-      </c>
-      <c r="I21" t="s">
-        <v>55</v>
-      </c>
-      <c r="J21" t="s">
-        <v>55</v>
-      </c>
-      <c r="K21" s="2"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22">
-        <f>SUM(D2:D21)</f>
+      <c r="D23">
+        <f>SUM(D3:D22)</f>
         <v>17</v>
       </c>
-      <c r="E22">
-        <f t="shared" ref="E22:J22" si="1">SUM(E2:E21)</f>
+      <c r="E23">
+        <f>SUM(E3:E22)</f>
         <v>8.75</v>
       </c>
-      <c r="F22">
-        <f t="shared" si="1"/>
+      <c r="F23">
+        <f>SUM(F3:F22)</f>
         <v>30</v>
       </c>
-      <c r="G22">
-        <f t="shared" si="1"/>
+      <c r="G23">
+        <f>SUM(G3:G22)</f>
         <v>12.75</v>
       </c>
-      <c r="H22">
-        <f t="shared" si="1"/>
+      <c r="H23">
+        <f>SUM(H3:H22)</f>
         <v>14.5</v>
       </c>
-      <c r="I22">
-        <f t="shared" si="1"/>
+      <c r="I23">
+        <f>SUM(I3:I22)</f>
         <v>16.25</v>
       </c>
-      <c r="J22">
-        <f t="shared" si="1"/>
+      <c r="J23">
+        <f>SUM(J3:J22)</f>
         <v>99.25</v>
       </c>
-      <c r="K22" s="2"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D23" s="1">
-        <f>SUM(D2:D21)/34</f>
-        <v>0.5</v>
-      </c>
-      <c r="E23" s="1">
-        <f>SUM(E2:E21)/34</f>
+      <c r="K23" s="2"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D24" s="1">
+        <f>SUM(D3:D22)/34</f>
+        <v>0.5</v>
+      </c>
+      <c r="E24" s="1">
+        <f>SUM(E3:E22)/34</f>
         <v>0.25735294117647056</v>
       </c>
-      <c r="F23" s="1">
-        <f>SUM(F2:F21)/34</f>
+      <c r="F24" s="1">
+        <f>SUM(F3:F22)/34</f>
         <v>0.88235294117647056</v>
       </c>
-      <c r="G23" s="1">
-        <f>SUM(G2:G21)/34</f>
+      <c r="G24" s="1">
+        <f>SUM(G3:G22)/34</f>
         <v>0.375</v>
       </c>
-      <c r="H23" s="1">
-        <f>SUM(H2:H21)/34</f>
+      <c r="H24" s="1">
+        <f>SUM(H3:H22)/34</f>
         <v>0.4264705882352941</v>
       </c>
-      <c r="I23" s="1">
-        <f>SUM(I2:I21)/34</f>
+      <c r="I24" s="1">
+        <f>SUM(I3:I22)/34</f>
         <v>0.47794117647058826</v>
       </c>
-      <c r="J23" s="1">
-        <f>SUM(J2:J21)/(34*6)</f>
+      <c r="J24" s="1">
+        <f>SUM(J3:J22)/(34*6)</f>
         <v>0.48651960784313725</v>
       </c>
-      <c r="K23" s="2"/>
+      <c r="K24" s="2"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J21">
-    <sortCondition ref="J2:J21"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:K24">
+    <sortCondition ref="C3:C24"/>
+    <sortCondition ref="B3:B24"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1448,8 +1452,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C470603-E249-6C49-AFDF-564C1138E589}">
-  <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
@@ -1467,7 +1471,7 @@
     <col min="14" max="14" width="5.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="D1" t="s">
         <v>21</v>
       </c>
@@ -1484,7 +1488,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -1524,52 +1528,59 @@
       <c r="N2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>39</v>
       </c>
       <c r="D3">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N3">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+        <v>9.75</v>
+      </c>
+      <c r="O3" s="2">
+        <f>N3/10</f>
+        <v>0.97499999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>7</v>
       </c>
@@ -1612,57 +1623,65 @@
       <c r="N4">
         <v>5.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O4" s="2">
+        <f t="shared" ref="O4:O22" si="0">N4/10</f>
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
         <v>39</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J5">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="N5">
-        <v>6.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+        <v>2.5</v>
+      </c>
+      <c r="O5" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>39</v>
@@ -1674,39 +1693,43 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="N6">
-        <v>9.75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+        <v>6.75</v>
+      </c>
+      <c r="O6" s="2">
+        <f t="shared" si="0"/>
+        <v>0.67500000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
@@ -1727,7 +1750,7 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -1744,8 +1767,12 @@
       <c r="N7">
         <v>9.75</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O7" s="2">
+        <f t="shared" si="0"/>
+        <v>0.97499999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1788,96 +1815,108 @@
       <c r="N8">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <v>0.5</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="J9">
         <v>1</v>
       </c>
       <c r="K9">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="N9">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+      <c r="O9" s="2">
+        <f t="shared" si="0"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
         <v>2</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
         <v>0.5</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>1</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="N10">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+        <v>4.5</v>
+      </c>
+      <c r="O10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>16</v>
       </c>
@@ -1920,34 +1959,38 @@
       <c r="N11">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
         <v>45</v>
       </c>
       <c r="D12">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1959,39 +2002,43 @@
         <v>1</v>
       </c>
       <c r="M12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12">
-        <v>8.25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+        <v>8.75</v>
+      </c>
+      <c r="O12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="F13">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
       <c r="I13">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -2003,13 +2050,17 @@
         <v>1</v>
       </c>
       <c r="M13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13">
-        <v>8.75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+        <v>8.25</v>
+      </c>
+      <c r="O13" s="2">
+        <f t="shared" si="0"/>
+        <v>0.82499999999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>20</v>
       </c>
@@ -2052,8 +2103,12 @@
       <c r="N14" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O14" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>17</v>
       </c>
@@ -2096,8 +2151,12 @@
       <c r="N15">
         <v>9.5</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O15" s="2">
+        <f t="shared" si="0"/>
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>11</v>
       </c>
@@ -2140,22 +2199,26 @@
       <c r="N16">
         <v>6.25</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O16" s="2">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="C17" t="s">
         <v>37</v>
       </c>
       <c r="D17">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -2167,39 +2230,43 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17">
         <v>0</v>
       </c>
       <c r="N17">
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+        <v>3.5</v>
+      </c>
+      <c r="O17" s="2">
+        <f t="shared" si="0"/>
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
         <v>37</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E18">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -2211,25 +2278,29 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+        <v>1.25</v>
+      </c>
+      <c r="O18" s="2">
+        <f t="shared" si="0"/>
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>9</v>
       </c>
@@ -2272,8 +2343,12 @@
       <c r="N19">
         <v>5.75</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O19" s="2">
+        <f t="shared" si="0"/>
+        <v>0.57499999999999996</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>10</v>
       </c>
@@ -2316,8 +2391,12 @@
       <c r="N20">
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O20" s="2">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>8</v>
       </c>
@@ -2360,8 +2439,12 @@
       <c r="N21">
         <v>5.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O21" s="2">
+        <f t="shared" si="0"/>
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4</v>
       </c>
@@ -2404,94 +2487,102 @@
       <c r="N22">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O22" s="2">
+        <f t="shared" si="0"/>
+        <v>0.32500000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
       <c r="D23">
-        <f t="shared" ref="D23:M23" si="0">SUM(D3:D22)</f>
+        <f>SUM(D3:D22)</f>
         <v>13</v>
       </c>
       <c r="E23">
-        <f t="shared" si="0"/>
+        <f>SUM(E3:E22)</f>
         <v>16</v>
       </c>
       <c r="F23">
-        <f t="shared" si="0"/>
+        <f>SUM(F3:F22)</f>
         <v>9.25</v>
       </c>
       <c r="G23">
-        <f t="shared" si="0"/>
+        <f>SUM(G3:G22)</f>
         <v>8.25</v>
       </c>
       <c r="H23">
-        <f t="shared" si="0"/>
+        <f>SUM(H3:H22)</f>
         <v>10</v>
       </c>
       <c r="I23">
-        <f t="shared" si="0"/>
+        <f>SUM(I3:I22)</f>
         <v>12.5</v>
       </c>
       <c r="J23">
-        <f t="shared" si="0"/>
+        <f>SUM(J3:J22)</f>
         <v>14</v>
       </c>
       <c r="K23">
-        <f t="shared" si="0"/>
+        <f>SUM(K3:K22)</f>
         <v>11.25</v>
       </c>
       <c r="L23">
-        <f t="shared" si="0"/>
+        <f>SUM(L3:L22)</f>
         <v>13.5</v>
       </c>
       <c r="M23">
-        <f t="shared" si="0"/>
+        <f>SUM(M3:M22)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="D24" s="1">
-        <f t="shared" ref="D24:M24" si="1">D23/19</f>
+        <f>D23/19</f>
         <v>0.68421052631578949</v>
       </c>
       <c r="E24" s="1">
-        <f t="shared" si="1"/>
+        <f>E23/19</f>
         <v>0.84210526315789469</v>
       </c>
       <c r="F24" s="1">
-        <f t="shared" si="1"/>
+        <f>F23/19</f>
         <v>0.48684210526315791</v>
       </c>
       <c r="G24" s="1">
-        <f t="shared" si="1"/>
+        <f>G23/19</f>
         <v>0.43421052631578949</v>
       </c>
       <c r="H24" s="1">
-        <f t="shared" si="1"/>
+        <f>H23/19</f>
         <v>0.52631578947368418</v>
       </c>
       <c r="I24" s="1">
-        <f t="shared" si="1"/>
+        <f>I23/19</f>
         <v>0.65789473684210531</v>
       </c>
       <c r="J24" s="1">
-        <f t="shared" si="1"/>
+        <f>J23/19</f>
         <v>0.73684210526315785</v>
       </c>
       <c r="K24" s="1">
-        <f t="shared" si="1"/>
+        <f>K23/19</f>
         <v>0.59210526315789469</v>
       </c>
       <c r="L24" s="1">
-        <f t="shared" si="1"/>
+        <f>L23/19</f>
         <v>0.71052631578947367</v>
       </c>
       <c r="M24" s="1">
-        <f t="shared" si="1"/>
+        <f>M23/19</f>
         <v>0.36842105263157893</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:N22">
-    <sortCondition ref="C3:C22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:N24">
+    <sortCondition ref="C3:C24"/>
+    <sortCondition ref="B3:B24"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3390,7 +3481,7 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
         <v>55</v>
@@ -3428,43 +3519,43 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C24">
-        <f>SUM(C4:C22)</f>
+        <f t="shared" ref="C24:I24" si="1">SUM(C4:C22)</f>
         <v>13</v>
       </c>
       <c r="D24">
-        <f>SUM(D4:D22)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="E24">
-        <f>SUM(E4:E22)</f>
+        <f t="shared" si="1"/>
         <v>9.25</v>
       </c>
       <c r="F24">
-        <f>SUM(F4:F22)</f>
+        <f t="shared" si="1"/>
         <v>8.25</v>
       </c>
       <c r="G24">
-        <f>SUM(G4:G22)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="H24">
-        <f>SUM(H4:H22)</f>
+        <f t="shared" si="1"/>
         <v>12.5</v>
       </c>
       <c r="I24">
-        <f>SUM(I4:I22)</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="J24" s="1">
-        <f t="shared" ref="D24:L25" si="1">J23/19</f>
+        <f t="shared" ref="D24:L25" si="2">J23/19</f>
         <v>0.59210526315789469</v>
       </c>
       <c r="K24" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.71052631578947367</v>
       </c>
       <c r="L24" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.36842105263157893</v>
       </c>
     </row>
@@ -3474,27 +3565,27 @@
         <v>0.68421052631578949</v>
       </c>
       <c r="D25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.84210526315789469</v>
       </c>
       <c r="E25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.48684210526315791</v>
       </c>
       <c r="F25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.43421052631578949</v>
       </c>
       <c r="G25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.52631578947368418</v>
       </c>
       <c r="H25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.65789473684210531</v>
       </c>
       <c r="I25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.73684210526315785</v>
       </c>
     </row>

</xml_diff>